<commit_message>
Actualización de documentación, incorporación de cambios a fecha (10/10/2026), actualización de 4.4 Docker
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/3.1 Criterios de Aceptación/CRITERIOS DE ACEPTACIÓN.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/3.1 Criterios de Aceptación/CRITERIOS DE ACEPTACIÓN.xlsx
@@ -13,10 +13,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={6f750d83-3f3e-4be5-a9a5-c4d6b738d35b}</author>
+    <author>tc={21b37613-1440-4023-a375-1c0e8e738cce}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{6f750d83-3f3e-4be5-a9a5-c4d6b738d35b}" ref="A1">
+    <comment authorId="0" xr:uid="{21b37613-1440-4023-a375-1c0e8e738cce}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -379,7 +379,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="ALONSO . GONZALEZ JARA" id="{f05ad8ee-abfd-4a3b-be5f-a205b7b3d676}" providerId="google-sheets"/>
+  <x18tc:person displayName="ALONSO . GONZALEZ JARA" id="{d4ce0fe2-2a16-4803-bdf1-7dfb65b964d9}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -579,7 +579,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A1" dT="2026-09-06T18:27:44.00" personId="{f05ad8ee-abfd-4a3b-be5f-a205b7b3d676}" id="{6f750d83-3f3e-4be5-a9a5-c4d6b738d35b}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-09-06T18:27:44.00" personId="{d4ce0fe2-2a16-4803-bdf1-7dfb65b964d9}" id="{21b37613-1440-4023-a375-1c0e8e738cce}" done="0">
     <x18tc:text xml:space="preserve">Hice la tabla en relación a los criterios de aceptación que se definieron en el product backlog</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>

</xml_diff>

<commit_message>
Incorporación de Cambios Documentales actuales a mi rama
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de documentación/3.1 Criterios de Aceptación/CRITERIOS DE ACEPTACIÓN.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de documentación/3.1 Criterios de Aceptación/CRITERIOS DE ACEPTACIÓN.xlsx
@@ -13,10 +13,10 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision">
   <authors>
-    <author>tc={21b37613-1440-4023-a375-1c0e8e738cce}</author>
+    <author>tc={bb7a9ee7-3d99-4776-88d4-c14d07edae97}</author>
   </authors>
   <commentList>
-    <comment authorId="0" xr:uid="{21b37613-1440-4023-a375-1c0e8e738cce}" ref="A1">
+    <comment authorId="0" xr:uid="{bb7a9ee7-3d99-4776-88d4-c14d07edae97}" ref="A1">
       <text>
         <t xml:space="preserve">[Threaded comment]
  Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -379,7 +379,7 @@
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments">
-  <x18tc:person displayName="ALONSO . GONZALEZ JARA" id="{d4ce0fe2-2a16-4803-bdf1-7dfb65b964d9}" providerId="google-sheets"/>
+  <x18tc:person displayName="ALONSO . GONZALEZ JARA" id="{00ba20f2-946a-4c41-bcef-8e655a60a68e}" providerId="google-sheets"/>
 </x18tc:personList>
 </file>
 
@@ -579,7 +579,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <x18tc:ThreadedComments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:xltc2="http://schemas.microsoft.com/office/spreadsheetml/2020/threadedcomments2" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <x18tc:threadedComment ref="A1" dT="2026-09-06T18:27:44.00" personId="{d4ce0fe2-2a16-4803-bdf1-7dfb65b964d9}" id="{21b37613-1440-4023-a375-1c0e8e738cce}" done="0">
+  <x18tc:threadedComment ref="A1" dT="2026-09-06T18:27:44.00" personId="{00ba20f2-946a-4c41-bcef-8e655a60a68e}" id="{bb7a9ee7-3d99-4776-88d4-c14d07edae97}" done="0">
     <x18tc:text xml:space="preserve">Hice la tabla en relación a los criterios de aceptación que se definieron en el product backlog</x18tc:text>
   </x18tc:threadedComment>
 </x18tc:ThreadedComments>
@@ -673,14 +673,20 @@
       <c r="B8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>23</v>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Validación de formato de número telefónico (E.164)</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>El número se normaliza y valida en formato E.164 (por ejemplo, +56 9 1234 5678; máximo 15 dígitos). No se permite registrar un número duplicado en la lista ni el número propio del usuario.</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>El campo muestra un error de validación, bloquea el botón de guardado y genera la notificación "El número telefónico ingresado no tiene un formato válido"</t>
+        </is>
       </c>
     </row>
     <row r="9" ht="89.25" customHeight="1">
@@ -727,11 +733,15 @@
       <c r="C11" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>37</v>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>El mensaje de emergencia personalizado del usuario tiene un máximo de 160 caracteres, validado en el frontend y en el backend.</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>La interfaz impide escribir más de 160 caracteres y muestra un contador que cambia a rojo al llegar al límite; el backend rechaza mensajes de más de 160 caracteres.</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="89.25" customHeight="1">
@@ -744,8 +754,10 @@
       <c r="C12" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="D12" s="6" t="s">
-        <v>41</v>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>La interfaz exige mantener presionado el botón SOS (o botón asignado) continuamente por 5 segundos para generar un llamado de emergencia en el perfil predeterminado de personas mayores o usuarios con acceso limitado; la duración es configurable según el tipo de usuario (valor para el resto de perfiles pendiente de confirmar)</t>
+        </is>
       </c>
       <c r="E12" s="6" t="s">
         <v>42</v>
@@ -778,11 +790,15 @@
       <c r="C14" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="D14" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>52</v>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>Por cada contacto asignado, el sistema registra al menos un intento de envío con su estado (PENDIENTE, ENVIADO o FALLIDO), número de intentos y hora exacta. El criterio se cumple cuando el 100 % de los contactos tiene un intento registrado y un estado final.</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Si un envío falla por problemas del proveedor, el sistema reintenta con espera incremental y registra el error por destinatario; el usuario ve cuántos contactos fueron notificados.</t>
+        </is>
       </c>
     </row>
     <row r="15" ht="108.0" customHeight="1">

</xml_diff>